<commit_message>
add logo in excel
</commit_message>
<xml_diff>
--- a/Result_Update_Layout.xlsx
+++ b/Result_Update_Layout.xlsx
@@ -33,8 +33,8 @@
   </si>
   <si>
     <t xml:space="preserve">โปรเจค : โซลาร์เซลล์ 10k 1เฟส 
-          กำลังไฟสูงสุด ( 10.00kWp ) 
-          INVERTER : HUAWEI 
+      กำลังไฟสูงสุด ( 10.00kWp ) 
+      INVERTER : HUAWEI 
  วันที่ : 13 / 5 / 2568 
  เลขที่เอกสาร : PNMMA25016</t>
   </si>
@@ -287,9 +287,9 @@
     <t>สองแสนสี่หมื่นสี่พันบาทถ้วน</t>
   </si>
   <si>
-    <t xml:space="preserve">ลงชื่อผู้ให้บริการ
-___________________
-วันที่ 13 / 5 / 2568</t>
+    <t xml:space="preserve">                                   ลงชื่อผู้ให้บริการ
+                                   ___________________
+                                   วันที่ 13 / 5 / 2568</t>
   </si>
   <si>
     <t xml:space="preserve">ลงชื่อลูกค้า
@@ -456,6 +456,94 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>10000</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2190750" cy="904875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2454,5 +2542,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>